<commit_message>
Add footer block, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files (13):
- blocks/footer/footer.css
- blocks/footer/footer.js
- footer.plain.html
- icons/facebook.svg
- icons/instagram.svg
- icons/linkedin.svg
- icons/tiktok.svg
- icons/x.svg
- icons/youtube.svg
- nav.plain.html
- tools/importer/import-story-article.bundle.js
- tools/importer/reports/import-story-article.report.xlsx
- tools/importer/transformers/abbvie-cleanup.js
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-story-article.report.xlsx
+++ b/tools/importer/reports/import-story-article.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="25">
   <si>
     <t>_reportFile</t>
   </si>
@@ -19,6 +19,12 @@
     <t>blocks</t>
   </si>
   <si>
+    <t>error</t>
+  </si>
+  <si>
+    <t>errorStack</t>
+  </si>
+  <si>
     <t>path</t>
   </si>
   <si>
@@ -37,6 +43,36 @@
     <t>url</t>
   </si>
   <si>
+    <t>who-we-are/our-stories/three-ways-ai-is-changing-drug-discovery-at-abbvie.html.report.json</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t xml:space="preserve">page.evaluate: Error: Failed to import page: metadataDiv is not defined
+    at eval (eval at evaluate (:290:30), &lt;anonymous&gt;:29:15)
+    at async &lt;anonymous&gt;:316:30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">page.evaluate: Error: Failed to import page: metadataDiv is not defined
+    at eval (eval at evaluate (:290:30), &lt;anonymous&gt;:29:15)
+    at async &lt;anonymous&gt;:316:30
+    at processUrl (/home/node/.excat-marketplace/excat/skills/excat-content-import/scripts/run-bulk-import.js:455:31)
+    at async main (/home/node/.excat-marketplace/excat/skills/excat-content-import/scripts/run-bulk-import.js:599:22)</t>
+  </si>
+  <si>
+    <t>who-we-are/our-stories/three-ways-ai-is-changing-drug-discovery-at-abbvie.html</t>
+  </si>
+  <si>
+    <t>failed</t>
+  </si>
+  <si>
+    <t>2026-05-27T19:52:42.204Z</t>
+  </si>
+  <si>
+    <t>https://www.abbvie.com/who-we-are/our-stories/three-ways-ai-is-changing-drug-discovery-at-abbvie.html</t>
+  </si>
+  <si>
     <t>who-we-are/our-stories/three-ways-ai-is-changing-drug-discovery-at-abbvie.report.json</t>
   </si>
   <si>
@@ -52,13 +88,10 @@
     <t>story-article</t>
   </si>
   <si>
-    <t>2026-05-27T19:33:38.535Z</t>
+    <t>2026-05-28T16:10:49.008Z</t>
   </si>
   <si>
     <t>Three ways AI is changing drug discovery at AbbVie | AbbVie</t>
-  </si>
-  <si>
-    <t>https://www.abbvie.com/who-we-are/our-stories/three-ways-ai-is-changing-drug-discovery-at-abbvie.html</t>
   </si>
 </sst>
 </file>
@@ -447,16 +480,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="3" width="50" customWidth="1"/>
-    <col min="5" max="5" width="15" customWidth="1"/>
-    <col min="6" max="6" width="26" customWidth="1"/>
-    <col min="7" max="8" width="50" customWidth="1"/>
+    <col min="1" max="5" width="50" customWidth="1"/>
+    <col min="7" max="7" width="15" customWidth="1"/>
+    <col min="8" max="8" width="26" customWidth="1"/>
+    <col min="9" max="10" width="50" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -481,35 +514,79 @@
       <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B2" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C2" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G2" t="s">
         <v>11</v>
       </c>
-      <c r="E2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G2" t="s">
-        <v>14</v>
-      </c>
       <c r="H2" t="s">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="I2" t="s">
+        <v>11</v>
+      </c>
+      <c r="J2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F3" t="s">
+        <v>21</v>
+      </c>
+      <c r="G3" t="s">
+        <v>22</v>
+      </c>
+      <c r="H3" t="s">
+        <v>23</v>
+      </c>
+      <c r="I3" t="s">
+        <v>24</v>
+      </c>
+      <c r="J3" t="s">
+        <v>17</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H1"/>
+  <autoFilter ref="A1:J1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>